<commit_message>
add generated requirements files to template
</commit_message>
<xml_diff>
--- a/lib/inferno/apps/cli/templates/lib/%library_name%/requirements/Inferno Requirements Template.xlsx
+++ b/lib/inferno/apps/cli/templates/lib/%library_name%/requirements/Inferno Requirements Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/knaden/Documents/Inferno/source/inferno-core/lib/inferno/apps/cli/templates/lib/%library_name%/requirements/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/inferno-core/lib/inferno/apps/cli/templates/lib/%library_name%/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027030A2-86B7-144D-82D2-9BC5810EC972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6551332-D0E3-2D42-AEA7-2BE7EB34DD02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="9" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="121">
   <si>
     <t>ID*</t>
   </si>
@@ -154,9 +154,6 @@
   </si>
   <si>
     <t>Server</t>
-  </si>
-  <si>
-    <t>&lt;req set id&gt;@#</t>
   </si>
   <si>
     <t>Yes</t>
@@ -720,6 +717,15 @@
 - when removing content, use an ellipsis (three periods) to indicate where it was removed, e.g., "Some superflous details were removed ... from the middle of this requirement".
 For example, when extracting requiremenst from the narrative text "The ice cream parlor SHALL sell ice cream in waffle cones. It SHALL also offer chocolate sprinkle toppings.", the "It" in the second sentence cannot stand alone and the word "also" only makes sense in the context of the first sentence, but is not needed if the second is standing alone. One way to represent the second sentence would be add context from the first setence and remove the superflous details using the syntax described above: "[The ice cream parlor] SHALL ...offer chocolate sprinkle toppings."</t>
   </si>
+  <si>
+    <t>sample_v1</t>
+  </si>
+  <si>
+    <t>sample_v1@13</t>
+  </si>
+  <si>
+    <t>This is a subsrequirement, and it SHOULD be implemented.</t>
+  </si>
 </sst>
 </file>
 
@@ -955,7 +961,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1004,12 +1010,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1034,22 +1034,13 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1057,6 +1048,18 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1397,428 +1400,424 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.33203125" style="16" customWidth="1"/>
-    <col min="2" max="2" width="133.5" style="39" customWidth="1"/>
-    <col min="3" max="3" width="52.5" style="39" customWidth="1"/>
+    <col min="2" max="2" width="133.5" style="21" customWidth="1"/>
+    <col min="3" max="3" width="52.5" style="21" customWidth="1"/>
     <col min="4" max="4" width="91.1640625" style="21" customWidth="1"/>
     <col min="5" max="16384" width="10.83203125" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="16"/>
+    </row>
+    <row r="2" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="39"/>
+      <c r="D2" s="16"/>
+    </row>
+    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A3" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="40"/>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="40"/>
+      <c r="D4" s="16"/>
+    </row>
+    <row r="5" spans="1:4" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="41" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="41"/>
+      <c r="D5" s="16"/>
+    </row>
+    <row r="6" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="16"/>
+    </row>
+    <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="40"/>
+      <c r="D7" s="16"/>
+    </row>
+    <row r="8" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A8" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="40"/>
+      <c r="D8" s="16"/>
+    </row>
+    <row r="9" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="16"/>
-    </row>
-    <row r="2" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="36" t="s">
-        <v>57</v>
-      </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="16"/>
-    </row>
-    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A3" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" s="37"/>
-      <c r="D3" s="16"/>
-    </row>
-    <row r="4" spans="1:4" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="37" t="s">
+      <c r="B9" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="40"/>
+      <c r="D9" s="16"/>
+    </row>
+    <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A10" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="40"/>
+      <c r="D10" s="16"/>
+    </row>
+    <row r="11" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="40" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="40"/>
+      <c r="D11" s="16"/>
+    </row>
+    <row r="12" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="16"/>
+    </row>
+    <row r="14" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A14" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="25"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" s="22"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="22"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="22"/>
+    </row>
+    <row r="18" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A18" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="22"/>
+    </row>
+    <row r="19" spans="1:4" ht="112" x14ac:dyDescent="0.2">
+      <c r="A19" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="22"/>
+    </row>
+    <row r="20" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A20" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="22"/>
+    </row>
+    <row r="21" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A21" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="22"/>
+    </row>
+    <row r="22" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A22" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D22" s="22"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="C23" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D23" s="22"/>
+    </row>
+    <row r="24" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A24" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D24" s="22"/>
+    </row>
+    <row r="25" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A25" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="22"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="30" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="29" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="16"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" s="16"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="16"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D32" s="16"/>
+    </row>
+    <row r="33" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A33" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D33" s="16"/>
+    </row>
+    <row r="34" spans="1:4" ht="22" x14ac:dyDescent="0.3">
+      <c r="A34" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B34" s="35"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="16"/>
+    </row>
+    <row r="35" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="C35" s="36"/>
+    </row>
+    <row r="36" spans="1:4" ht="134" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="34" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="37"/>
-      <c r="D4" s="16"/>
-    </row>
-    <row r="5" spans="1:4" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="38"/>
-      <c r="D5" s="16"/>
-    </row>
-    <row r="6" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="16"/>
-    </row>
-    <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="37" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="37"/>
-      <c r="D7" s="16"/>
-    </row>
-    <row r="8" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A8" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="37" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="37"/>
-      <c r="D8" s="16"/>
-    </row>
-    <row r="9" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="16"/>
-    </row>
-    <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="B10" s="37" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="16"/>
-    </row>
-    <row r="11" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="B11" s="37" t="s">
+      <c r="B36" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="38"/>
+    </row>
+    <row r="37" spans="1:4" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="34" t="s">
         <v>108</v>
       </c>
-      <c r="C11" s="37"/>
-      <c r="D11" s="16"/>
-    </row>
-    <row r="12" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D13" s="16"/>
-    </row>
-    <row r="14" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A14" s="33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B14" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="D14" s="25"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="30" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" s="22"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="B16" s="30" t="s">
-        <v>81</v>
-      </c>
-      <c r="C16" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="D16" s="22"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="30" t="s">
-        <v>83</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="D17" s="22"/>
-    </row>
-    <row r="18" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A18" s="33" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="D18" s="22"/>
-    </row>
-    <row r="19" spans="1:4" ht="112" x14ac:dyDescent="0.2">
-      <c r="A19" s="33" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="D19" s="22"/>
-    </row>
-    <row r="20" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A20" s="33" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20" s="22"/>
-    </row>
-    <row r="21" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A21" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="B21" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="C21" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="D21" s="22"/>
-    </row>
-    <row r="22" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A22" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D22" s="22"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D23" s="22"/>
-    </row>
-    <row r="24" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A24" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="C24" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D24" s="22"/>
-    </row>
-    <row r="25" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A25" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="B25" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="C25" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D25" s="22"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="B26" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="C26" s="32" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="35" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="C27" s="32" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="34" t="s">
-        <v>14</v>
-      </c>
-      <c r="B28" s="31" t="s">
-        <v>102</v>
-      </c>
-      <c r="C28" s="31" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="34" t="s">
-        <v>101</v>
-      </c>
-      <c r="B29" s="31" t="s">
-        <v>103</v>
-      </c>
-      <c r="C29" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="D29" s="16"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="34" t="s">
-        <v>16</v>
-      </c>
-      <c r="B30" s="31" t="s">
-        <v>104</v>
-      </c>
-      <c r="C30" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="D30" s="16"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="B31" s="31" t="s">
-        <v>105</v>
-      </c>
-      <c r="C31" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="D31" s="16"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="34" t="s">
-        <v>18</v>
-      </c>
-      <c r="B32" s="31" t="s">
-        <v>106</v>
-      </c>
-      <c r="C32" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="D32" s="16"/>
-    </row>
-    <row r="33" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A33" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="B33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="C33" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="D33" s="16"/>
-    </row>
-    <row r="34" spans="1:4" ht="22" x14ac:dyDescent="0.3">
-      <c r="A34" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="16"/>
-    </row>
-    <row r="35" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="41" t="s">
-        <v>114</v>
-      </c>
-      <c r="B35" s="40" t="s">
-        <v>113</v>
-      </c>
-      <c r="C35" s="40"/>
-    </row>
-    <row r="36" spans="1:4" ht="134" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="41" t="s">
-        <v>117</v>
-      </c>
-      <c r="B36" s="42" t="s">
-        <v>118</v>
-      </c>
-      <c r="C36" s="43"/>
-    </row>
-    <row r="37" spans="1:4" ht="112" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="41" t="s">
+      <c r="B37" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="36"/>
+      <c r="D37" s="16"/>
+    </row>
+    <row r="38" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="B37" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="C37" s="40"/>
-      <c r="D37" s="16"/>
-    </row>
-    <row r="38" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="41" t="s">
+      <c r="B38" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="B38" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="C38" s="40"/>
+      <c r="C38" s="36"/>
       <c r="D38" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1830,7 +1829,11 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B36:C36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1945,22 +1948,22 @@
       <c r="E2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>24</v>
+      <c r="F2" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="G2" s="7" t="b">
         <v>0</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" s="8" t="s">
         <v>26</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>27</v>
       </c>
       <c r="M2" s="9" t="str" cm="1">
         <f t="array" ref="M2">PAGE_NAME(B2)</f>
@@ -1982,25 +1985,41 @@
       <c r="AD2" s="14"/>
     </row>
     <row r="3" spans="1:36" s="5" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="A3" s="7">
+        <v>13</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="F3" s="8"/>
-      <c r="G3" s="7"/>
+      <c r="G3" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="H3" s="10"/>
-      <c r="I3" s="8"/>
+      <c r="I3" s="8" t="s">
+        <v>24</v>
+      </c>
       <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
+      <c r="K3" s="8" t="s">
+        <v>24</v>
+      </c>
       <c r="L3" s="8"/>
       <c r="M3" s="9" t="str" cm="1">
         <f t="array" ref="M3">PAGE_NAME(B3)</f>
-        <v/>
+        <v>page</v>
       </c>
       <c r="N3" s="9" t="str" cm="1">
         <f t="array" ref="N3">SECTION_NAME(B3)</f>
-        <v/>
+        <v>section</v>
       </c>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
@@ -5533,6 +5552,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{D8959B40-E618-764F-B8D3-E9A5190F88A4}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -5571,68 +5593,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B1" s="26"/>
+      <c r="A1" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="42"/>
     </row>
     <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
+      <c r="A2" s="42"/>
+      <c r="B2" s="42"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -5654,19 +5679,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B1" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="D1" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="E1" s="19" t="s">
         <v>41</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -5674,13 +5699,13 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>44</v>
-      </c>
-      <c r="D2" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -5695,13 +5720,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
         <v>6</v>
       </c>
       <c r="C1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D1" t="s">
         <v>8</v>
@@ -5715,47 +5740,47 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="b">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" t="s">
         <v>51</v>
-      </c>
-      <c r="C4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -5764,6 +5789,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -6017,15 +6051,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6040,6 +6065,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E19681A-8DD3-40CB-9262-8533E89B98A6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6059,14 +6092,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
   <ds:schemaRefs>

</xml_diff>